<commit_message>
Agregar script de instalacion de LibreOffice
</commit_message>
<xml_diff>
--- a/Inventario_Inteligente_ImportBolts.xlsx
+++ b/Inventario_Inteligente_ImportBolts.xlsx
@@ -1,20 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Victor\Desktop\SistemaAnclajes\PruebaDespiegue\sistemaANCLAJES\sistema-importbolts-main\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A354C472-2AE7-453B-B7D4-88982AC9EA67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="138">
   <si>
     <t>CÓDIGO</t>
   </si>
@@ -413,13 +424,28 @@
   </si>
   <si>
     <t>F.N</t>
+  </si>
+  <si>
+    <t>ESTADO</t>
+  </si>
+  <si>
+    <t>OXIDADO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">POR REPASAR </t>
+  </si>
+  <si>
+    <t>FALTA PINTAR</t>
+  </si>
+  <si>
+    <t>ROTOS</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -482,13 +508,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -526,7 +560,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -560,6 +594,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -594,9 +629,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -769,11 +805,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J46"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:K46"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="8.88671875" customWidth="1"/>
+    <col min="2" max="2" width="45.77734375" customWidth="1"/>
+    <col min="3" max="3" width="29.44140625" customWidth="1"/>
+    <col min="4" max="4" width="19.44140625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -781,31 +823,34 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -813,28 +858,31 @@
         <v>55</v>
       </c>
       <c r="C2" t="s">
+        <v>134</v>
+      </c>
+      <c r="D2" t="s">
         <v>89</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>92</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>131</v>
       </c>
-      <c r="F2">
+      <c r="G2">
         <v>2527</v>
       </c>
-      <c r="G2">
-        <v>10</v>
-      </c>
       <c r="H2">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I2">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:10">
+      <c r="J2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -842,57 +890,60 @@
         <v>56</v>
       </c>
       <c r="C3" t="s">
+        <v>135</v>
+      </c>
+      <c r="D3" t="s">
         <v>90</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>93</v>
       </c>
-      <c r="E3" t="s">
-        <v>132</v>
-      </c>
-      <c r="F3">
+      <c r="F3" t="s">
+        <v>132</v>
+      </c>
+      <c r="G3">
         <v>2049</v>
       </c>
-      <c r="G3">
-        <v>10</v>
-      </c>
       <c r="H3">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I3">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:10">
+      <c r="J3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>12</v>
       </c>
       <c r="B4" t="s">
         <v>57</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>90</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>94</v>
       </c>
-      <c r="E4" t="s">
-        <v>132</v>
-      </c>
-      <c r="F4">
+      <c r="F4" t="s">
+        <v>132</v>
+      </c>
+      <c r="G4">
         <v>2025</v>
       </c>
-      <c r="G4">
-        <v>10</v>
-      </c>
       <c r="H4">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I4">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:10">
+      <c r="J4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -900,115 +951,118 @@
         <v>58</v>
       </c>
       <c r="C5" t="s">
+        <v>136</v>
+      </c>
+      <c r="D5" t="s">
         <v>90</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>95</v>
       </c>
-      <c r="E5" t="s">
-        <v>132</v>
-      </c>
-      <c r="F5">
+      <c r="F5" t="s">
+        <v>132</v>
+      </c>
+      <c r="G5">
         <v>1014</v>
       </c>
-      <c r="G5">
-        <v>10</v>
-      </c>
       <c r="H5">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I5">
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:10">
+      <c r="J5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>14</v>
       </c>
       <c r="B6" t="s">
         <v>59</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>90</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>96</v>
       </c>
-      <c r="E6" t="s">
-        <v>132</v>
-      </c>
-      <c r="F6">
+      <c r="F6" t="s">
+        <v>132</v>
+      </c>
+      <c r="G6">
         <v>995</v>
       </c>
-      <c r="G6">
-        <v>10</v>
-      </c>
       <c r="H6">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I6">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:10">
+      <c r="J6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>15</v>
       </c>
       <c r="B7" t="s">
         <v>60</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>90</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>97</v>
       </c>
-      <c r="E7" t="s">
-        <v>132</v>
-      </c>
-      <c r="F7">
+      <c r="F7" t="s">
+        <v>132</v>
+      </c>
+      <c r="G7">
         <v>1001</v>
       </c>
-      <c r="G7">
-        <v>10</v>
-      </c>
       <c r="H7">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I7">
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:10">
+      <c r="J7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>16</v>
       </c>
       <c r="B8" t="s">
         <v>61</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>90</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>98</v>
       </c>
-      <c r="E8" t="s">
-        <v>132</v>
-      </c>
-      <c r="F8">
+      <c r="F8" t="s">
+        <v>132</v>
+      </c>
+      <c r="G8">
         <v>1037</v>
       </c>
-      <c r="G8">
-        <v>10</v>
-      </c>
       <c r="H8">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I8">
         <v>0</v>
       </c>
-    </row>
-    <row r="9" spans="1:10">
+      <c r="J8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>17</v>
       </c>
@@ -1016,1097 +1070,1100 @@
         <v>62</v>
       </c>
       <c r="C9" t="s">
+        <v>137</v>
+      </c>
+      <c r="D9" t="s">
         <v>90</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>99</v>
       </c>
-      <c r="E9" t="s">
-        <v>132</v>
-      </c>
-      <c r="F9">
+      <c r="F9" t="s">
+        <v>132</v>
+      </c>
+      <c r="G9">
         <v>1049</v>
       </c>
-      <c r="G9">
-        <v>10</v>
-      </c>
       <c r="H9">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I9">
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:10">
+      <c r="J9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>18</v>
       </c>
       <c r="B10" t="s">
         <v>63</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
         <v>90</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>100</v>
       </c>
-      <c r="E10" t="s">
-        <v>132</v>
-      </c>
-      <c r="F10">
+      <c r="F10" t="s">
+        <v>132</v>
+      </c>
+      <c r="G10">
         <v>995</v>
       </c>
-      <c r="G10">
-        <v>10</v>
-      </c>
       <c r="H10">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I10">
         <v>0</v>
       </c>
-    </row>
-    <row r="11" spans="1:10">
+      <c r="J10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>19</v>
       </c>
       <c r="B11" t="s">
         <v>64</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" t="s">
         <v>90</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>101</v>
       </c>
-      <c r="E11" t="s">
-        <v>132</v>
-      </c>
-      <c r="F11">
+      <c r="F11" t="s">
+        <v>132</v>
+      </c>
+      <c r="G11">
         <v>994</v>
       </c>
-      <c r="G11">
-        <v>10</v>
-      </c>
       <c r="H11">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I11">
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:10">
+      <c r="J11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>20</v>
       </c>
       <c r="B12" t="s">
         <v>65</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
         <v>90</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
         <v>102</v>
       </c>
-      <c r="E12" t="s">
-        <v>132</v>
-      </c>
-      <c r="F12">
+      <c r="F12" t="s">
+        <v>132</v>
+      </c>
+      <c r="G12">
         <v>1000</v>
       </c>
-      <c r="G12">
-        <v>10</v>
-      </c>
       <c r="H12">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I12">
         <v>0</v>
       </c>
-    </row>
-    <row r="13" spans="1:10">
+      <c r="J12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>21</v>
       </c>
       <c r="B13" t="s">
         <v>66</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
         <v>90</v>
       </c>
-      <c r="D13" t="s">
+      <c r="E13" t="s">
         <v>103</v>
       </c>
-      <c r="E13" t="s">
-        <v>132</v>
-      </c>
-      <c r="F13">
+      <c r="F13" t="s">
+        <v>132</v>
+      </c>
+      <c r="G13">
         <v>1487</v>
       </c>
-      <c r="G13">
-        <v>10</v>
-      </c>
       <c r="H13">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I13">
         <v>0</v>
       </c>
-    </row>
-    <row r="14" spans="1:10">
+      <c r="J13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>22</v>
       </c>
       <c r="B14" t="s">
         <v>67</v>
       </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
         <v>90</v>
       </c>
-      <c r="D14" t="s">
+      <c r="E14" t="s">
         <v>96</v>
       </c>
-      <c r="E14" t="s">
-        <v>132</v>
-      </c>
-      <c r="F14">
+      <c r="F14" t="s">
+        <v>132</v>
+      </c>
+      <c r="G14">
         <v>1345</v>
       </c>
-      <c r="G14">
-        <v>10</v>
-      </c>
       <c r="H14">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I14">
         <v>0</v>
       </c>
-    </row>
-    <row r="15" spans="1:10">
+      <c r="J14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>23</v>
       </c>
       <c r="B15" t="s">
         <v>68</v>
       </c>
-      <c r="C15" t="s">
+      <c r="D15" t="s">
         <v>90</v>
       </c>
-      <c r="D15" t="s">
+      <c r="E15" t="s">
         <v>96</v>
       </c>
-      <c r="E15" t="s">
-        <v>132</v>
-      </c>
-      <c r="F15">
+      <c r="F15" t="s">
+        <v>132</v>
+      </c>
+      <c r="G15">
         <v>2608</v>
       </c>
-      <c r="G15">
-        <v>10</v>
-      </c>
       <c r="H15">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I15">
         <v>0</v>
       </c>
-    </row>
-    <row r="16" spans="1:10">
+      <c r="J15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>24</v>
       </c>
       <c r="B16" t="s">
         <v>69</v>
       </c>
-      <c r="C16" t="s">
+      <c r="D16" t="s">
         <v>90</v>
       </c>
-      <c r="D16" t="s">
+      <c r="E16" t="s">
         <v>104</v>
       </c>
-      <c r="E16" t="s">
-        <v>132</v>
-      </c>
-      <c r="F16">
+      <c r="F16" t="s">
+        <v>132</v>
+      </c>
+      <c r="G16">
         <v>2410</v>
       </c>
-      <c r="G16">
-        <v>10</v>
-      </c>
       <c r="H16">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I16">
         <v>0</v>
       </c>
-    </row>
-    <row r="17" spans="1:9">
+      <c r="J16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>25</v>
       </c>
       <c r="B17" t="s">
         <v>70</v>
       </c>
-      <c r="C17" t="s">
+      <c r="D17" t="s">
         <v>90</v>
       </c>
-      <c r="D17" t="s">
+      <c r="E17" t="s">
         <v>105</v>
       </c>
-      <c r="E17" t="s">
-        <v>132</v>
-      </c>
-      <c r="F17">
+      <c r="F17" t="s">
+        <v>132</v>
+      </c>
+      <c r="G17">
         <v>2271</v>
       </c>
-      <c r="G17">
-        <v>10</v>
-      </c>
       <c r="H17">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I17">
         <v>0</v>
       </c>
-    </row>
-    <row r="18" spans="1:9">
+      <c r="J17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>26</v>
       </c>
       <c r="B18" t="s">
         <v>71</v>
       </c>
-      <c r="C18" t="s">
+      <c r="D18" t="s">
         <v>90</v>
       </c>
-      <c r="D18" t="s">
+      <c r="E18" t="s">
         <v>96</v>
       </c>
-      <c r="E18" t="s">
-        <v>132</v>
-      </c>
-      <c r="F18">
+      <c r="F18" t="s">
+        <v>132</v>
+      </c>
+      <c r="G18">
         <v>1900</v>
       </c>
-      <c r="G18">
-        <v>10</v>
-      </c>
       <c r="H18">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I18">
         <v>0</v>
       </c>
-    </row>
-    <row r="19" spans="1:9">
+      <c r="J18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>27</v>
       </c>
       <c r="B19" t="s">
         <v>72</v>
       </c>
-      <c r="C19" t="s">
+      <c r="D19" t="s">
         <v>90</v>
       </c>
-      <c r="D19" t="s">
+      <c r="E19" t="s">
         <v>96</v>
       </c>
-      <c r="E19" t="s">
-        <v>132</v>
-      </c>
-      <c r="F19">
+      <c r="F19" t="s">
+        <v>132</v>
+      </c>
+      <c r="G19">
         <v>1324</v>
       </c>
-      <c r="G19">
-        <v>10</v>
-      </c>
       <c r="H19">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I19">
         <v>0</v>
       </c>
-    </row>
-    <row r="20" spans="1:9">
+      <c r="J19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>28</v>
       </c>
       <c r="B20" t="s">
         <v>73</v>
       </c>
-      <c r="C20" t="s">
+      <c r="D20" t="s">
         <v>90</v>
       </c>
-      <c r="D20" t="s">
+      <c r="E20" t="s">
         <v>106</v>
       </c>
-      <c r="E20" t="s">
-        <v>132</v>
-      </c>
-      <c r="F20">
+      <c r="F20" t="s">
+        <v>132</v>
+      </c>
+      <c r="G20">
         <v>2038</v>
       </c>
-      <c r="G20">
-        <v>10</v>
-      </c>
       <c r="H20">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I20">
         <v>0</v>
       </c>
-    </row>
-    <row r="21" spans="1:9">
+      <c r="J20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>29</v>
       </c>
       <c r="B21" t="s">
         <v>74</v>
       </c>
-      <c r="C21" t="s">
+      <c r="D21" t="s">
         <v>90</v>
       </c>
-      <c r="D21" t="s">
+      <c r="E21" t="s">
         <v>107</v>
       </c>
-      <c r="E21" t="s">
-        <v>132</v>
-      </c>
-      <c r="F21">
+      <c r="F21" t="s">
+        <v>132</v>
+      </c>
+      <c r="G21">
         <v>2019</v>
       </c>
-      <c r="G21">
-        <v>10</v>
-      </c>
       <c r="H21">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I21">
         <v>0</v>
       </c>
-    </row>
-    <row r="22" spans="1:9">
+      <c r="J21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>30</v>
       </c>
       <c r="B22" t="s">
         <v>75</v>
       </c>
-      <c r="C22" t="s">
+      <c r="D22" t="s">
         <v>90</v>
       </c>
-      <c r="D22" t="s">
+      <c r="E22" t="s">
         <v>108</v>
       </c>
-      <c r="E22" t="s">
-        <v>132</v>
-      </c>
-      <c r="F22">
+      <c r="F22" t="s">
+        <v>132</v>
+      </c>
+      <c r="G22">
         <v>1151</v>
       </c>
-      <c r="G22">
-        <v>10</v>
-      </c>
       <c r="H22">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I22">
         <v>0</v>
       </c>
-    </row>
-    <row r="23" spans="1:9">
+      <c r="J22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>31</v>
       </c>
       <c r="B23" t="s">
         <v>76</v>
       </c>
-      <c r="C23" t="s">
+      <c r="D23" t="s">
         <v>90</v>
       </c>
-      <c r="D23" t="s">
+      <c r="E23" t="s">
         <v>96</v>
       </c>
-      <c r="E23" t="s">
-        <v>132</v>
-      </c>
-      <c r="F23">
+      <c r="F23" t="s">
+        <v>132</v>
+      </c>
+      <c r="G23">
         <v>994</v>
       </c>
-      <c r="G23">
-        <v>10</v>
-      </c>
       <c r="H23">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I23">
         <v>0</v>
       </c>
-    </row>
-    <row r="24" spans="1:9">
+      <c r="J23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>32</v>
       </c>
       <c r="B24" t="s">
         <v>77</v>
       </c>
-      <c r="C24" t="s">
+      <c r="D24" t="s">
         <v>90</v>
       </c>
-      <c r="D24" t="s">
+      <c r="E24" t="s">
         <v>109</v>
       </c>
-      <c r="E24" t="s">
-        <v>132</v>
-      </c>
-      <c r="F24">
+      <c r="F24" t="s">
+        <v>132</v>
+      </c>
+      <c r="G24">
         <v>1000</v>
       </c>
-      <c r="G24">
-        <v>10</v>
-      </c>
       <c r="H24">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I24">
         <v>0</v>
       </c>
-    </row>
-    <row r="25" spans="1:9">
+      <c r="J24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>33</v>
       </c>
       <c r="B25" t="s">
         <v>78</v>
       </c>
-      <c r="C25" t="s">
+      <c r="D25" t="s">
         <v>91</v>
       </c>
-      <c r="D25" t="s">
+      <c r="E25" t="s">
         <v>110</v>
       </c>
-      <c r="E25" t="s">
+      <c r="F25" t="s">
         <v>131</v>
       </c>
-      <c r="F25">
+      <c r="G25">
         <v>6020</v>
       </c>
-      <c r="G25">
-        <v>10</v>
-      </c>
       <c r="H25">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I25">
         <v>0</v>
       </c>
-    </row>
-    <row r="26" spans="1:9">
+      <c r="J25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>34</v>
       </c>
       <c r="B26" t="s">
         <v>79</v>
       </c>
-      <c r="C26" t="s">
+      <c r="D26" t="s">
         <v>91</v>
       </c>
-      <c r="D26" t="s">
+      <c r="E26" t="s">
         <v>111</v>
       </c>
-      <c r="E26" t="s">
+      <c r="F26" t="s">
         <v>131</v>
       </c>
-      <c r="F26">
+      <c r="G26">
         <v>1015</v>
       </c>
-      <c r="G26">
-        <v>10</v>
-      </c>
       <c r="H26">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I26">
         <v>0</v>
       </c>
-    </row>
-    <row r="27" spans="1:9">
+      <c r="J26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>35</v>
       </c>
       <c r="B27" t="s">
         <v>80</v>
       </c>
-      <c r="C27" t="s">
+      <c r="D27" t="s">
         <v>91</v>
       </c>
-      <c r="D27" t="s">
+      <c r="E27" t="s">
         <v>112</v>
       </c>
-      <c r="E27" t="s">
+      <c r="F27" t="s">
         <v>131</v>
       </c>
-      <c r="F27">
+      <c r="G27">
         <v>5131</v>
       </c>
-      <c r="G27">
-        <v>10</v>
-      </c>
       <c r="H27">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I27">
         <v>0</v>
       </c>
-    </row>
-    <row r="28" spans="1:9">
+      <c r="J27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>36</v>
       </c>
       <c r="B28" t="s">
         <v>81</v>
       </c>
-      <c r="C28" t="s">
+      <c r="D28" t="s">
         <v>91</v>
       </c>
-      <c r="D28" t="s">
+      <c r="E28" t="s">
         <v>113</v>
       </c>
-      <c r="E28" t="s">
+      <c r="F28" t="s">
         <v>131</v>
       </c>
-      <c r="F28">
+      <c r="G28">
         <v>5339</v>
       </c>
-      <c r="G28">
-        <v>10</v>
-      </c>
       <c r="H28">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I28">
         <v>0</v>
       </c>
-    </row>
-    <row r="29" spans="1:9">
+      <c r="J28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>37</v>
       </c>
       <c r="B29" t="s">
         <v>82</v>
       </c>
-      <c r="C29" t="s">
+      <c r="D29" t="s">
         <v>91</v>
       </c>
-      <c r="D29" t="s">
+      <c r="E29" t="s">
         <v>114</v>
       </c>
-      <c r="E29" t="s">
+      <c r="F29" t="s">
         <v>131</v>
       </c>
-      <c r="F29">
+      <c r="G29">
         <v>75533</v>
       </c>
-      <c r="G29">
-        <v>10</v>
-      </c>
       <c r="H29">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I29">
         <v>0</v>
       </c>
-    </row>
-    <row r="30" spans="1:9">
+      <c r="J29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>38</v>
       </c>
       <c r="B30" t="s">
         <v>83</v>
       </c>
-      <c r="C30" t="s">
+      <c r="D30" t="s">
         <v>91</v>
       </c>
-      <c r="D30" t="s">
+      <c r="E30" t="s">
         <v>115</v>
       </c>
-      <c r="E30" t="s">
+      <c r="F30" t="s">
         <v>131</v>
       </c>
-      <c r="F30">
+      <c r="G30">
         <v>1103</v>
       </c>
-      <c r="G30">
-        <v>10</v>
-      </c>
       <c r="H30">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I30">
         <v>0</v>
       </c>
-    </row>
-    <row r="31" spans="1:9">
+      <c r="J30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>39</v>
       </c>
       <c r="B31" t="s">
         <v>84</v>
       </c>
-      <c r="C31" t="s">
+      <c r="D31" t="s">
         <v>91</v>
       </c>
-      <c r="D31" t="s">
+      <c r="E31" t="s">
         <v>96</v>
       </c>
-      <c r="E31" t="s">
+      <c r="F31" t="s">
         <v>131</v>
       </c>
-      <c r="F31">
+      <c r="G31">
         <v>1018</v>
       </c>
-      <c r="G31">
-        <v>10</v>
-      </c>
       <c r="H31">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I31">
         <v>0</v>
       </c>
-    </row>
-    <row r="32" spans="1:9">
+      <c r="J31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>40</v>
       </c>
       <c r="B32" t="s">
         <v>85</v>
       </c>
-      <c r="C32" t="s">
+      <c r="D32" t="s">
         <v>91</v>
       </c>
-      <c r="D32" t="s">
+      <c r="E32" t="s">
         <v>116</v>
       </c>
-      <c r="E32" t="s">
+      <c r="F32" t="s">
         <v>131</v>
       </c>
-      <c r="F32">
+      <c r="G32">
         <v>1017</v>
       </c>
-      <c r="G32">
-        <v>10</v>
-      </c>
       <c r="H32">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I32">
         <v>0</v>
       </c>
-    </row>
-    <row r="33" spans="1:9">
+      <c r="J32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>41</v>
       </c>
       <c r="B33" t="s">
         <v>86</v>
       </c>
-      <c r="C33" t="s">
+      <c r="D33" t="s">
         <v>91</v>
       </c>
-      <c r="D33" t="s">
+      <c r="E33" t="s">
         <v>117</v>
       </c>
-      <c r="E33" t="s">
+      <c r="F33" t="s">
         <v>131</v>
       </c>
-      <c r="F33">
+      <c r="G33">
         <v>52491</v>
       </c>
-      <c r="G33">
-        <v>10</v>
-      </c>
       <c r="H33">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I33">
         <v>0</v>
       </c>
-    </row>
-    <row r="34" spans="1:9">
+      <c r="J33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>42</v>
       </c>
       <c r="B34" t="s">
         <v>87</v>
       </c>
-      <c r="C34" t="s">
+      <c r="D34" t="s">
         <v>91</v>
       </c>
-      <c r="D34" t="s">
+      <c r="E34" t="s">
         <v>118</v>
       </c>
-      <c r="E34" t="s">
+      <c r="F34" t="s">
         <v>131</v>
       </c>
-      <c r="F34">
+      <c r="G34">
         <v>87132</v>
       </c>
-      <c r="G34">
-        <v>10</v>
-      </c>
       <c r="H34">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I34">
         <v>0</v>
       </c>
-    </row>
-    <row r="35" spans="1:9">
+      <c r="J34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>43</v>
       </c>
       <c r="B35" t="s">
         <v>88</v>
       </c>
-      <c r="C35" t="s">
+      <c r="D35" t="s">
         <v>91</v>
       </c>
-      <c r="D35" t="s">
+      <c r="E35" t="s">
         <v>119</v>
       </c>
-      <c r="E35" t="s">
+      <c r="F35" t="s">
         <v>131</v>
       </c>
-      <c r="F35">
+      <c r="G35">
         <v>5840</v>
       </c>
-      <c r="G35">
-        <v>10</v>
-      </c>
       <c r="H35">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I35">
         <v>0</v>
       </c>
-    </row>
-    <row r="36" spans="1:9">
+      <c r="J35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>44</v>
       </c>
       <c r="B36" t="s">
         <v>78</v>
       </c>
-      <c r="C36" t="s">
+      <c r="D36" t="s">
         <v>91</v>
       </c>
-      <c r="D36" t="s">
+      <c r="E36" t="s">
         <v>120</v>
       </c>
-      <c r="E36" t="s">
-        <v>132</v>
-      </c>
-      <c r="F36">
+      <c r="F36" t="s">
+        <v>132</v>
+      </c>
+      <c r="G36">
         <v>10080</v>
       </c>
-      <c r="G36">
-        <v>10</v>
-      </c>
       <c r="H36">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I36">
         <v>0</v>
       </c>
-    </row>
-    <row r="37" spans="1:9">
+      <c r="J36">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>45</v>
       </c>
       <c r="B37" t="s">
         <v>79</v>
       </c>
-      <c r="C37" t="s">
+      <c r="D37" t="s">
         <v>91</v>
       </c>
-      <c r="D37" t="s">
+      <c r="E37" t="s">
         <v>121</v>
       </c>
-      <c r="E37" t="s">
-        <v>132</v>
-      </c>
-      <c r="F37">
+      <c r="F37" t="s">
+        <v>132</v>
+      </c>
+      <c r="G37">
         <v>2079</v>
       </c>
-      <c r="G37">
-        <v>10</v>
-      </c>
       <c r="H37">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I37">
         <v>0</v>
       </c>
-    </row>
-    <row r="38" spans="1:9">
+      <c r="J37">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>46</v>
       </c>
       <c r="B38" t="s">
         <v>80</v>
       </c>
-      <c r="C38" t="s">
+      <c r="D38" t="s">
         <v>91</v>
       </c>
-      <c r="D38" t="s">
+      <c r="E38" t="s">
         <v>122</v>
       </c>
-      <c r="E38" t="s">
-        <v>132</v>
-      </c>
-      <c r="F38">
+      <c r="F38" t="s">
+        <v>132</v>
+      </c>
+      <c r="G38">
         <v>5142</v>
       </c>
-      <c r="G38">
-        <v>10</v>
-      </c>
       <c r="H38">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I38">
         <v>0</v>
       </c>
-    </row>
-    <row r="39" spans="1:9">
+      <c r="J38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>47</v>
       </c>
       <c r="B39" t="s">
         <v>81</v>
       </c>
-      <c r="C39" t="s">
+      <c r="D39" t="s">
         <v>91</v>
       </c>
-      <c r="D39" t="s">
+      <c r="E39" t="s">
         <v>123</v>
       </c>
-      <c r="E39" t="s">
-        <v>132</v>
-      </c>
-      <c r="F39">
+      <c r="F39" t="s">
+        <v>132</v>
+      </c>
+      <c r="G39">
         <v>5665</v>
       </c>
-      <c r="G39">
-        <v>10</v>
-      </c>
       <c r="H39">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I39">
         <v>0</v>
       </c>
-    </row>
-    <row r="40" spans="1:9">
+      <c r="J39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>48</v>
       </c>
       <c r="B40" t="s">
         <v>82</v>
       </c>
-      <c r="C40" t="s">
+      <c r="D40" t="s">
         <v>91</v>
       </c>
-      <c r="D40" t="s">
+      <c r="E40" t="s">
         <v>124</v>
       </c>
-      <c r="E40" t="s">
-        <v>132</v>
-      </c>
-      <c r="F40">
+      <c r="F40" t="s">
+        <v>132</v>
+      </c>
+      <c r="G40">
         <v>71089</v>
       </c>
-      <c r="G40">
-        <v>10</v>
-      </c>
       <c r="H40">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I40">
         <v>0</v>
       </c>
-    </row>
-    <row r="41" spans="1:9">
+      <c r="J40">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>49</v>
       </c>
       <c r="B41" t="s">
         <v>83</v>
       </c>
-      <c r="C41" t="s">
+      <c r="D41" t="s">
         <v>91</v>
       </c>
-      <c r="D41" t="s">
+      <c r="E41" t="s">
         <v>125</v>
       </c>
-      <c r="E41" t="s">
-        <v>132</v>
-      </c>
-      <c r="F41">
+      <c r="F41" t="s">
+        <v>132</v>
+      </c>
+      <c r="G41">
         <v>1191</v>
       </c>
-      <c r="G41">
-        <v>10</v>
-      </c>
       <c r="H41">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I41">
         <v>0</v>
       </c>
-    </row>
-    <row r="42" spans="1:9">
+      <c r="J41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>50</v>
       </c>
       <c r="B42" t="s">
         <v>84</v>
       </c>
-      <c r="C42" t="s">
+      <c r="D42" t="s">
         <v>91</v>
       </c>
-      <c r="D42" t="s">
+      <c r="E42" t="s">
         <v>126</v>
       </c>
-      <c r="E42" t="s">
-        <v>132</v>
-      </c>
-      <c r="F42">
+      <c r="F42" t="s">
+        <v>132</v>
+      </c>
+      <c r="G42">
         <v>2074</v>
       </c>
-      <c r="G42">
-        <v>10</v>
-      </c>
       <c r="H42">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I42">
         <v>0</v>
       </c>
-    </row>
-    <row r="43" spans="1:9">
+      <c r="J42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>51</v>
       </c>
       <c r="B43" t="s">
         <v>85</v>
       </c>
-      <c r="C43" t="s">
+      <c r="D43" t="s">
         <v>91</v>
       </c>
-      <c r="D43" t="s">
+      <c r="E43" t="s">
         <v>127</v>
       </c>
-      <c r="E43" t="s">
-        <v>132</v>
-      </c>
-      <c r="F43">
+      <c r="F43" t="s">
+        <v>132</v>
+      </c>
+      <c r="G43">
         <v>1073</v>
       </c>
-      <c r="G43">
-        <v>10</v>
-      </c>
       <c r="H43">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I43">
         <v>0</v>
       </c>
-    </row>
-    <row r="44" spans="1:9">
+      <c r="J43">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>52</v>
       </c>
       <c r="B44" t="s">
         <v>86</v>
       </c>
-      <c r="C44" t="s">
+      <c r="D44" t="s">
         <v>91</v>
       </c>
-      <c r="D44" t="s">
+      <c r="E44" t="s">
         <v>128</v>
       </c>
-      <c r="E44" t="s">
-        <v>132</v>
-      </c>
-      <c r="F44">
+      <c r="F44" t="s">
+        <v>132</v>
+      </c>
+      <c r="G44">
         <v>20100</v>
       </c>
-      <c r="G44">
-        <v>10</v>
-      </c>
       <c r="H44">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I44">
         <v>0</v>
       </c>
-    </row>
-    <row r="45" spans="1:9">
+      <c r="J44">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>53</v>
       </c>
       <c r="B45" t="s">
         <v>87</v>
       </c>
-      <c r="C45" t="s">
+      <c r="D45" t="s">
         <v>91</v>
       </c>
-      <c r="D45" t="s">
+      <c r="E45" t="s">
         <v>129</v>
       </c>
-      <c r="E45" t="s">
-        <v>132</v>
-      </c>
-      <c r="F45">
+      <c r="F45" t="s">
+        <v>132</v>
+      </c>
+      <c r="G45">
         <v>20000</v>
       </c>
-      <c r="G45">
-        <v>10</v>
-      </c>
       <c r="H45">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I45">
         <v>0</v>
       </c>
-    </row>
-    <row r="46" spans="1:9">
+      <c r="J45">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>54</v>
       </c>
       <c r="B46" t="s">
         <v>88</v>
       </c>
-      <c r="C46" t="s">
+      <c r="D46" t="s">
         <v>91</v>
       </c>
-      <c r="D46" t="s">
+      <c r="E46" t="s">
         <v>130</v>
       </c>
-      <c r="E46" t="s">
-        <v>132</v>
-      </c>
-      <c r="F46">
+      <c r="F46" t="s">
+        <v>132</v>
+      </c>
+      <c r="G46">
         <v>5348</v>
       </c>
-      <c r="G46">
-        <v>10</v>
-      </c>
       <c r="H46">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I46">
+        <v>0</v>
+      </c>
+      <c r="J46">
         <v>0</v>
       </c>
     </row>

</xml_diff>